<commit_message>
feat: sort solutions by station order, hard delete, and fix status cell editor
- Sort solutions by Station.sort_order in Solution Map, Data Management,
  G$ Management, and Excel export
- Change delete solution from soft delete to hard delete (removes solution_map
  entries and document files)
- Fix StatusCellEditor to allow creating new solution_map entries for empty cells
  (previously Save button was disabled when no existing status)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TC Finishing D^t Solution Migration_2026.xlsx
+++ b/TC Finishing D^t Solution Migration_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://corningonline-my.sharepoint.com/personal/wangm44_corning_com/Documents/桌面/Project/Dt_Quality_Roadmap/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangm44\Project\Dt_Quality_Roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="515" documentId="14_{89C73AE1-523B-4B10-8D61-849337C2FCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1BB2A86-7869-4B1B-95BD-A204095BBA20}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0546802D-6A1B-44CD-8B46-512262E44C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Definition" sheetId="6" r:id="rId1"/>
@@ -963,9 +963,6 @@
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
   <si>
-    <t>Tilter/SA TAM sensor</t>
-  </si>
-  <si>
     <t>N/A</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
@@ -1897,6 +1894,10 @@
   </si>
   <si>
     <t>BKG detection system; Wet zone glass BKG detective system; Cell grinder BKG detection system at OUT C/V</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>TAM sensor</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
@@ -2640,6 +2641,7 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2670,7 +2672,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -3599,7 +3600,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>13</v>
@@ -3632,182 +3633,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="64" t="s">
-        <v>329</v>
-      </c>
-      <c r="C1" s="64" t="s">
+      <c r="B1" s="54" t="s">
+        <v>328</v>
+      </c>
+      <c r="C1" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="64" t="s">
+      <c r="D1" s="54" t="s">
         <v>162</v>
       </c>
-      <c r="E1" s="64" t="s">
-        <v>440</v>
-      </c>
-      <c r="F1" s="64" t="s">
-        <v>406</v>
+      <c r="E1" s="54" t="s">
+        <v>439</v>
+      </c>
+      <c r="F1" s="54" t="s">
+        <v>405</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C3" t="s">
+        <v>312</v>
+      </c>
+      <c r="D3" t="s">
         <v>313</v>
       </c>
-      <c r="D3" t="s">
-        <v>314</v>
-      </c>
       <c r="E3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="F4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E5" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D6" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E6" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B7" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E7" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D8" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="E8" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F8" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B9" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C9" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D9" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E9" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C10" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E10" t="s">
         <v>205</v>
@@ -3815,397 +3816,397 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B11" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C11" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D11" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="E11" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F11" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B12" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C12" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D12" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E12" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="F12" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B13" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C13" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D13" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E13" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B14" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D14" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="E14" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="F14" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B15" t="s">
+        <v>332</v>
+      </c>
+      <c r="C15" t="s">
         <v>333</v>
       </c>
-      <c r="C15" t="s">
-        <v>334</v>
-      </c>
       <c r="D15" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E15" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B16" t="s">
+        <v>332</v>
+      </c>
+      <c r="C16" t="s">
         <v>333</v>
       </c>
-      <c r="C16" t="s">
-        <v>334</v>
-      </c>
       <c r="D16" t="s">
+        <v>444</v>
+      </c>
+      <c r="E16" t="s">
         <v>445</v>
       </c>
-      <c r="E16" t="s">
-        <v>446</v>
-      </c>
       <c r="F16" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B17" t="s">
+        <v>332</v>
+      </c>
+      <c r="C17" t="s">
         <v>333</v>
       </c>
-      <c r="C17" t="s">
-        <v>334</v>
-      </c>
       <c r="D17" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E17" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B18" t="s">
+        <v>332</v>
+      </c>
+      <c r="C18" t="s">
         <v>333</v>
       </c>
-      <c r="C18" t="s">
-        <v>334</v>
-      </c>
       <c r="D18" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E18" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B19" t="s">
+        <v>332</v>
+      </c>
+      <c r="C19" t="s">
         <v>333</v>
       </c>
-      <c r="C19" t="s">
-        <v>334</v>
-      </c>
       <c r="D19" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E19" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B20" t="s">
+        <v>332</v>
+      </c>
+      <c r="C20" t="s">
         <v>333</v>
       </c>
-      <c r="C20" t="s">
-        <v>334</v>
-      </c>
       <c r="D20" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E20" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B21" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C21" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D21" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E21" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B22" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C22" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D22" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E22" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B23" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C23" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D23" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E23" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B24" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C24" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D24" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E24" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="F24" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B25" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C25" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D25" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E25" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="F25" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B26" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D26" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E26" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B27" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C27" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D27" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E27" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="F27" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B28" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C28" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D28" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E28" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B29" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C29" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="D29" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E29" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F29" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B30" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C30" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D30" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E30" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B31" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C31" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D31" t="s">
         <v>187</v>
       </c>
       <c r="E31" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B32" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C32" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D32" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E32" t="s">
         <v>205</v>
@@ -4216,7 +4217,7 @@
         <v>99</v>
       </c>
       <c r="B33" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C33" t="s">
         <v>164</v>
@@ -4233,19 +4234,19 @@
         <v>99</v>
       </c>
       <c r="B34" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C34" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D34" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E34" t="s">
         <v>205</v>
       </c>
       <c r="F34" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -4253,13 +4254,13 @@
         <v>99</v>
       </c>
       <c r="B35" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C35" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D35" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -4267,13 +4268,13 @@
         <v>99</v>
       </c>
       <c r="B36" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C36" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D36" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -4281,16 +4282,16 @@
         <v>99</v>
       </c>
       <c r="B37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C37" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D37" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="E37" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -4298,16 +4299,16 @@
         <v>99</v>
       </c>
       <c r="B38" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C38" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D38" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E38" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -4315,16 +4316,16 @@
         <v>99</v>
       </c>
       <c r="B39" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C39" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D39" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E39" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -4332,16 +4333,16 @@
         <v>99</v>
       </c>
       <c r="B40" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C40" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D40" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E40" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -4349,13 +4350,13 @@
         <v>99</v>
       </c>
       <c r="B41" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C41" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D41" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E41" t="s">
         <v>205</v>
@@ -4366,13 +4367,13 @@
         <v>99</v>
       </c>
       <c r="B42" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C42" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D42" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E42" t="s">
         <v>205</v>
@@ -4383,10 +4384,10 @@
         <v>99</v>
       </c>
       <c r="B43" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C43" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -4394,10 +4395,10 @@
         <v>99</v>
       </c>
       <c r="B44" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C44" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -4405,19 +4406,19 @@
         <v>99</v>
       </c>
       <c r="B45" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C45" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D45" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E45" t="s">
         <v>205</v>
       </c>
       <c r="F45" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -4425,19 +4426,19 @@
         <v>99</v>
       </c>
       <c r="B46" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D46" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E46" t="s">
         <v>219</v>
       </c>
       <c r="F46" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -4445,13 +4446,13 @@
         <v>99</v>
       </c>
       <c r="B47" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C47" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D47" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -4459,16 +4460,16 @@
         <v>99</v>
       </c>
       <c r="B48" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C48" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D48" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E48" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -4476,19 +4477,19 @@
         <v>99</v>
       </c>
       <c r="B49" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C49" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D49" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E49" t="s">
         <v>219</v>
       </c>
       <c r="F49" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -4496,10 +4497,10 @@
         <v>99</v>
       </c>
       <c r="B50" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C50" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -4507,10 +4508,10 @@
         <v>99</v>
       </c>
       <c r="B51" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C51" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -4518,10 +4519,10 @@
         <v>99</v>
       </c>
       <c r="B52" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C52" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -4529,10 +4530,10 @@
         <v>99</v>
       </c>
       <c r="B53" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -4540,10 +4541,10 @@
         <v>99</v>
       </c>
       <c r="B54" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C54" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -4551,19 +4552,19 @@
         <v>99</v>
       </c>
       <c r="B55" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C55" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D55" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E55" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="F55" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -4571,16 +4572,16 @@
         <v>99</v>
       </c>
       <c r="B56" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C56" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D56" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E56" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -4588,16 +4589,16 @@
         <v>99</v>
       </c>
       <c r="B57" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C57" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D57" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E57" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -4605,16 +4606,16 @@
         <v>99</v>
       </c>
       <c r="B58" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C58" t="s">
         <v>176</v>
       </c>
       <c r="D58" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E58" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -4622,7 +4623,7 @@
         <v>99</v>
       </c>
       <c r="B59" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C59" t="s">
         <v>178</v>
@@ -4631,7 +4632,7 @@
         <v>175</v>
       </c>
       <c r="E59" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -4639,16 +4640,16 @@
         <v>99</v>
       </c>
       <c r="B60" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C60" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D60" t="s">
         <v>179</v>
       </c>
       <c r="E60" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -4656,10 +4657,10 @@
         <v>99</v>
       </c>
       <c r="B61" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C61" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -4667,16 +4668,16 @@
         <v>99</v>
       </c>
       <c r="B62" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C62" t="s">
         <v>181</v>
       </c>
       <c r="D62" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E62" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -4684,10 +4685,10 @@
         <v>99</v>
       </c>
       <c r="B63" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C63" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -4695,16 +4696,16 @@
         <v>99</v>
       </c>
       <c r="B64" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C64" t="s">
+        <v>419</v>
+      </c>
+      <c r="D64" t="s">
         <v>420</v>
       </c>
-      <c r="D64" t="s">
-        <v>421</v>
-      </c>
       <c r="E64" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -4721,7 +4722,7 @@
         <v>182</v>
       </c>
       <c r="E65" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -4735,13 +4736,13 @@
         <v>183</v>
       </c>
       <c r="D66" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E66" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F66" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -4752,16 +4753,16 @@
         <v>180</v>
       </c>
       <c r="C67" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D67" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E67" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F67" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -4772,10 +4773,10 @@
         <v>180</v>
       </c>
       <c r="C68" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D68" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="E68" t="s">
         <v>205</v>
@@ -4792,13 +4793,13 @@
         <v>185</v>
       </c>
       <c r="D69" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E69" t="s">
         <v>205</v>
       </c>
       <c r="F69" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -4815,7 +4816,7 @@
         <v>187</v>
       </c>
       <c r="E70" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -4829,13 +4830,13 @@
         <v>185</v>
       </c>
       <c r="D71" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E71" t="s">
         <v>205</v>
       </c>
       <c r="F71" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -4849,13 +4850,13 @@
         <v>185</v>
       </c>
       <c r="D72" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E72" t="s">
         <v>205</v>
       </c>
       <c r="F72" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -4872,7 +4873,7 @@
         <v>189</v>
       </c>
       <c r="E73" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -4886,10 +4887,10 @@
         <v>185</v>
       </c>
       <c r="D74" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E74" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -4900,16 +4901,16 @@
         <v>180</v>
       </c>
       <c r="C75" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D75" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E75" t="s">
         <v>205</v>
       </c>
       <c r="F75" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -4920,135 +4921,135 @@
         <v>180</v>
       </c>
       <c r="C76" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="D76" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E76" t="s">
         <v>205</v>
       </c>
       <c r="F76" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B77" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C77" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D77" t="s">
         <v>226</v>
       </c>
       <c r="E77" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B78" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C78" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D78" t="s">
         <v>85</v>
       </c>
       <c r="E78" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B79" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C79" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D79" t="s">
         <v>87</v>
       </c>
       <c r="E79" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B80" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C80" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D80" t="s">
         <v>88</v>
       </c>
       <c r="E80" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B81" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C81" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D81" t="s">
         <v>89</v>
       </c>
       <c r="E81" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B82" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C82" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D82" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E82" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B83" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C83" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D83" t="s">
         <v>171</v>
       </c>
       <c r="E83" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
   </sheetData>
@@ -6287,10 +6288,10 @@
         <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D1" t="s">
         <v>19</v>
@@ -6302,141 +6303,141 @@
         <v>80</v>
       </c>
       <c r="G1" t="s">
+        <v>248</v>
+      </c>
+      <c r="H1" t="s">
         <v>249</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>250</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>251</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>252</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>253</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>254</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>255</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>256</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>257</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>258</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>259</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>260</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>261</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>262</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>263</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>264</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>265</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>266</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>267</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>268</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>269</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>270</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>271</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>272</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>273</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>274</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>275</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>276</v>
       </c>
       <c r="AI1" t="s">
         <v>81</v>
       </c>
       <c r="AJ1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="AK1" t="s">
         <v>82</v>
       </c>
       <c r="AL1" t="s">
+        <v>277</v>
+      </c>
+      <c r="AM1" t="s">
         <v>278</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>279</v>
       </c>
       <c r="AN1" t="s">
         <v>83</v>
       </c>
       <c r="AO1" t="s">
+        <v>279</v>
+      </c>
+      <c r="AP1" t="s">
         <v>280</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>281</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>282</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>283</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>284</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>285</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B2" t="s">
         <v>287</v>
       </c>
-      <c r="B2" t="s">
-        <v>288</v>
-      </c>
       <c r="C2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E2" t="s">
         <v>2</v>
@@ -6570,16 +6571,16 @@
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E3" t="s">
         <v>8</v>
@@ -6713,16 +6714,16 @@
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B4" t="s">
         <v>287</v>
       </c>
-      <c r="B4" t="s">
-        <v>288</v>
-      </c>
       <c r="C4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="E4" t="s">
         <v>2</v>
@@ -6856,16 +6857,16 @@
     </row>
     <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>286</v>
+      </c>
+      <c r="B5" t="s">
         <v>287</v>
       </c>
-      <c r="B5" t="s">
-        <v>288</v>
-      </c>
       <c r="C5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D5" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E5" t="s">
         <v>8</v>
@@ -6999,16 +7000,16 @@
     </row>
     <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>286</v>
+      </c>
+      <c r="B6" t="s">
         <v>287</v>
       </c>
-      <c r="B6" t="s">
-        <v>288</v>
-      </c>
       <c r="C6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D6" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
@@ -7142,16 +7143,16 @@
     </row>
     <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>286</v>
+      </c>
+      <c r="B7" t="s">
         <v>287</v>
       </c>
-      <c r="B7" t="s">
-        <v>288</v>
-      </c>
       <c r="C7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E7" t="s">
         <v>14</v>
@@ -7285,16 +7286,16 @@
     </row>
     <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>286</v>
+      </c>
+      <c r="B8" t="s">
         <v>287</v>
       </c>
-      <c r="B8" t="s">
-        <v>288</v>
-      </c>
       <c r="C8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D8" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E8" t="s">
         <v>4</v>
@@ -7428,30 +7429,30 @@
     </row>
     <row r="9" spans="1:47" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>294</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>286</v>
+      </c>
+      <c r="B10" t="s">
         <v>287</v>
       </c>
-      <c r="B10" t="s">
-        <v>288</v>
-      </c>
       <c r="C10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D10" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E10" t="s">
         <v>2</v>
@@ -7585,16 +7586,16 @@
     </row>
     <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>286</v>
+      </c>
+      <c r="B11" t="s">
         <v>287</v>
       </c>
-      <c r="B11" t="s">
-        <v>288</v>
-      </c>
       <c r="C11" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D11" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E11" t="s">
         <v>14</v>
@@ -7728,16 +7729,16 @@
     </row>
     <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>286</v>
+      </c>
+      <c r="B12" t="s">
         <v>287</v>
       </c>
-      <c r="B12" t="s">
-        <v>288</v>
-      </c>
       <c r="C12" t="s">
+        <v>298</v>
+      </c>
+      <c r="D12" t="s">
         <v>299</v>
-      </c>
-      <c r="D12" t="s">
-        <v>300</v>
       </c>
       <c r="E12" t="s">
         <v>14</v>
@@ -7871,30 +7872,30 @@
     </row>
     <row r="13" spans="1:47" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>288</v>
-      </c>
       <c r="C13" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>286</v>
+      </c>
+      <c r="B14" t="s">
         <v>287</v>
       </c>
-      <c r="B14" t="s">
-        <v>288</v>
-      </c>
       <c r="C14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D14" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E14" t="s">
         <v>2</v>
@@ -8028,16 +8029,16 @@
     </row>
     <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>286</v>
+      </c>
+      <c r="B15" t="s">
         <v>287</v>
       </c>
-      <c r="B15" t="s">
-        <v>288</v>
-      </c>
       <c r="C15" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D15" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E15" t="s">
         <v>14</v>
@@ -8171,16 +8172,16 @@
     </row>
     <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>286</v>
+      </c>
+      <c r="B16" t="s">
         <v>287</v>
       </c>
-      <c r="B16" t="s">
-        <v>288</v>
-      </c>
       <c r="C16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D16" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E16" t="s">
         <v>2</v>
@@ -8314,16 +8315,16 @@
     </row>
     <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>286</v>
+      </c>
+      <c r="B17" t="s">
         <v>287</v>
       </c>
-      <c r="B17" t="s">
-        <v>288</v>
-      </c>
       <c r="C17" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D17" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E17" t="s">
         <v>2</v>
@@ -8457,16 +8458,16 @@
     </row>
     <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>286</v>
+      </c>
+      <c r="B18" t="s">
         <v>287</v>
       </c>
-      <c r="B18" t="s">
-        <v>288</v>
-      </c>
       <c r="C18" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D18" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -8600,16 +8601,16 @@
     </row>
     <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>286</v>
+      </c>
+      <c r="B19" t="s">
         <v>287</v>
       </c>
-      <c r="B19" t="s">
-        <v>288</v>
-      </c>
       <c r="C19" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D19" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E19" t="s">
         <v>14</v>
@@ -8743,16 +8744,16 @@
     </row>
     <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>286</v>
+      </c>
+      <c r="B20" t="s">
         <v>287</v>
       </c>
-      <c r="B20" t="s">
-        <v>288</v>
-      </c>
       <c r="C20" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D20" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E20" t="s">
         <v>2</v>
@@ -8886,16 +8887,16 @@
     </row>
     <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>286</v>
+      </c>
+      <c r="B21" t="s">
         <v>287</v>
       </c>
-      <c r="B21" t="s">
-        <v>288</v>
-      </c>
       <c r="C21" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D21" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E21" t="s">
         <v>14</v>
@@ -9029,30 +9030,30 @@
     </row>
     <row r="22" spans="1:47" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>288</v>
-      </c>
       <c r="C22" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B23" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C23" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D23" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E23" t="s">
         <v>4</v>
@@ -9186,16 +9187,16 @@
     </row>
     <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B24" t="s">
+        <v>311</v>
+      </c>
+      <c r="C24" t="s">
         <v>312</v>
       </c>
-      <c r="C24" t="s">
-        <v>313</v>
-      </c>
       <c r="D24" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E24" t="s">
         <v>2</v>
@@ -9329,16 +9330,16 @@
     </row>
     <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B25" t="s">
+        <v>311</v>
+      </c>
+      <c r="C25" t="s">
         <v>312</v>
       </c>
-      <c r="C25" t="s">
-        <v>313</v>
-      </c>
       <c r="D25" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E25" t="s">
         <v>4</v>
@@ -9472,16 +9473,16 @@
     </row>
     <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B26" t="s">
+        <v>311</v>
+      </c>
+      <c r="C26" t="s">
         <v>312</v>
       </c>
-      <c r="C26" t="s">
-        <v>313</v>
-      </c>
       <c r="D26" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E26" t="s">
         <v>4</v>
@@ -9615,16 +9616,16 @@
     </row>
     <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B27" t="s">
+        <v>311</v>
+      </c>
+      <c r="C27" t="s">
         <v>312</v>
       </c>
-      <c r="C27" t="s">
-        <v>313</v>
-      </c>
       <c r="D27" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -9758,16 +9759,16 @@
     </row>
     <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B28" t="s">
+        <v>311</v>
+      </c>
+      <c r="C28" t="s">
         <v>312</v>
       </c>
-      <c r="C28" t="s">
-        <v>313</v>
-      </c>
       <c r="D28" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E28" t="s">
         <v>14</v>
@@ -9901,16 +9902,16 @@
     </row>
     <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B29" t="s">
+        <v>311</v>
+      </c>
+      <c r="C29" t="s">
         <v>312</v>
       </c>
-      <c r="C29" t="s">
-        <v>313</v>
-      </c>
       <c r="D29" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E29" t="s">
         <v>14</v>
@@ -10044,16 +10045,16 @@
     </row>
     <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B30" t="s">
+        <v>311</v>
+      </c>
+      <c r="C30" t="s">
         <v>312</v>
       </c>
-      <c r="C30" t="s">
-        <v>313</v>
-      </c>
       <c r="D30" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E30" t="s">
         <v>14</v>
@@ -10187,16 +10188,16 @@
     </row>
     <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B31" t="s">
+        <v>311</v>
+      </c>
+      <c r="C31" t="s">
         <v>312</v>
       </c>
-      <c r="C31" t="s">
-        <v>313</v>
-      </c>
       <c r="D31" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="E31" t="s">
         <v>4</v>
@@ -10330,16 +10331,16 @@
     </row>
     <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B32" t="s">
+        <v>311</v>
+      </c>
+      <c r="C32" t="s">
         <v>312</v>
       </c>
-      <c r="C32" t="s">
-        <v>313</v>
-      </c>
       <c r="D32" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E32" t="s">
         <v>2</v>
@@ -10473,16 +10474,16 @@
     </row>
     <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B33" t="s">
+        <v>311</v>
+      </c>
+      <c r="C33" t="s">
         <v>312</v>
       </c>
-      <c r="C33" t="s">
-        <v>313</v>
-      </c>
       <c r="D33" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E33" t="s">
         <v>4</v>
@@ -10616,16 +10617,16 @@
     </row>
     <row r="34" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B34" t="s">
+        <v>311</v>
+      </c>
+      <c r="C34" t="s">
         <v>312</v>
       </c>
-      <c r="C34" t="s">
-        <v>313</v>
-      </c>
       <c r="D34" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E34" t="s">
         <v>14</v>
@@ -10759,16 +10760,16 @@
     </row>
     <row r="35" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B35" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C35" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D35" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E35" t="s">
         <v>4</v>
@@ -10902,16 +10903,16 @@
     </row>
     <row r="36" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B36" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C36" t="s">
+        <v>324</v>
+      </c>
+      <c r="D36" t="s">
         <v>325</v>
-      </c>
-      <c r="D36" t="s">
-        <v>326</v>
       </c>
       <c r="E36" t="s">
         <v>12</v>
@@ -11418,7 +11419,7 @@
         <v>95</v>
       </c>
       <c r="B2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C2" t="s">
         <v>97</v>
@@ -12188,7 +12189,7 @@
         <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E6" t="s">
         <v>86</v>
@@ -13331,7 +13332,7 @@
         <v>96</v>
       </c>
       <c r="C12" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D12" t="s">
         <v>111</v>
@@ -14098,7 +14099,7 @@
         <v>116</v>
       </c>
       <c r="D16" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E16" t="s">
         <v>86</v>
@@ -14113,7 +14114,7 @@
         <v>8</v>
       </c>
       <c r="I16" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J16" t="s">
         <v>10</v>
@@ -14289,7 +14290,7 @@
         <v>116</v>
       </c>
       <c r="D17" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E17" t="s">
         <v>86</v>
@@ -14480,7 +14481,7 @@
         <v>116</v>
       </c>
       <c r="D18" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E18" t="s">
         <v>86</v>
@@ -14671,7 +14672,7 @@
         <v>116</v>
       </c>
       <c r="D19" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="E19" t="s">
         <v>86</v>
@@ -14932,7 +14933,7 @@
         <v>96</v>
       </c>
       <c r="C21" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D21" t="s">
         <v>123</v>
@@ -19769,36 +19770,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="62" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="54" t="s">
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="55" t="s">
         <v>193</v>
       </c>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="55"/>
-      <c r="O1" s="55"/>
-      <c r="P1" s="55"/>
-      <c r="Q1" s="55"/>
-      <c r="R1" s="55"/>
-      <c r="S1" s="55"/>
-      <c r="T1" s="55"/>
-      <c r="U1" s="55"/>
-      <c r="V1" s="55"/>
-      <c r="W1" s="55"/>
-      <c r="X1" s="55"/>
-      <c r="Y1" s="56"/>
-      <c r="Z1" s="59" t="s">
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="56"/>
+      <c r="S1" s="56"/>
+      <c r="T1" s="56"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="56"/>
+      <c r="W1" s="56"/>
+      <c r="X1" s="56"/>
+      <c r="Y1" s="57"/>
+      <c r="Z1" s="60" t="s">
         <v>194</v>
       </c>
       <c r="AA1" s="27"/>
@@ -19817,28 +19818,28 @@
         <v>195</v>
       </c>
       <c r="E2" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="F2" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="G2" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="H2" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="I2" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="J2" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="K2" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="L2" s="10" t="s">
         <v>238</v>
-      </c>
-      <c r="L2" s="10" t="s">
-        <v>239</v>
       </c>
       <c r="M2" s="10" t="s">
         <v>44</v>
@@ -19847,7 +19848,7 @@
         <v>45</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P2" s="10" t="s">
         <v>47</v>
@@ -19859,19 +19860,19 @@
         <v>49</v>
       </c>
       <c r="S2" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="T2" s="10" t="s">
         <v>51</v>
       </c>
       <c r="U2" s="10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="V2" s="10" t="s">
         <v>53</v>
       </c>
       <c r="W2" s="10" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="X2" s="10" t="s">
         <v>55</v>
@@ -19879,7 +19880,7 @@
       <c r="Y2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="Z2" s="60"/>
+      <c r="Z2" s="61"/>
       <c r="AA2" s="28"/>
       <c r="AB2" s="8" t="s">
         <v>196</v>
@@ -19905,7 +19906,7 @@
         <v>163</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C3" s="47" t="s">
         <v>168</v>
@@ -20428,10 +20429,10 @@
         <v>132</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>174</v>
+        <v>400</v>
       </c>
       <c r="C16" s="47" t="s">
-        <v>228</v>
+        <v>481</v>
       </c>
       <c r="D16" s="39" t="s">
         <v>211</v>
@@ -20544,49 +20545,49 @@
         <v>216</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G18" s="20" t="s">
         <v>209</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I18" s="20" t="s">
         <v>209</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="N18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="O18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="P18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="Q18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="R18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="S18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="T18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="U18" s="20" t="s">
         <v>209</v>
@@ -20658,7 +20659,7 @@
         <v>157</v>
       </c>
       <c r="D20" s="46" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E20" s="42" t="s">
         <v>208</v>
@@ -20735,7 +20736,7 @@
         <v>157</v>
       </c>
       <c r="D21" s="46" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E21" s="12"/>
       <c r="F21" s="7"/>
@@ -20953,7 +20954,7 @@
         <v>189</v>
       </c>
       <c r="D25" s="39" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E25" s="18" t="s">
         <v>208</v>
@@ -21030,7 +21031,7 @@
         <v>157</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E26" s="44"/>
       <c r="F26" s="44"/>
@@ -21087,7 +21088,7 @@
         <v>157</v>
       </c>
       <c r="D27" s="46" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E27" s="12"/>
       <c r="F27" s="7"/>
@@ -21132,7 +21133,7 @@
         <v>226</v>
       </c>
       <c r="D28" s="40" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E28" s="30" t="s">
         <v>209</v>
@@ -21183,11 +21184,11 @@
       <c r="AA28" s="29"/>
     </row>
     <row r="29" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="57" t="s">
+      <c r="A29" s="58" t="s">
         <v>227</v>
       </c>
-      <c r="B29" s="58"/>
-      <c r="C29" s="58"/>
+      <c r="B29" s="59"/>
+      <c r="C29" s="59"/>
       <c r="D29" s="23"/>
       <c r="E29" s="24">
         <v>3</v>
@@ -21257,12 +21258,12 @@
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="E31" s="6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="E32" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -21400,7 +21401,7 @@
         <v>116</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -21431,7 +21432,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>99</v>
       </c>
@@ -21442,7 +21443,7 @@
         <v>110</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -21551,7 +21552,7 @@
         <v>132</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>179</v>

</xml_diff>